<commit_message>
chore: regenerate smoke xlsx to reflect 5-sheet structure
</commit_message>
<xml_diff>
--- a/reports/plans/noirs-boxes/2026-W19/2026-W19-0504-0510.xlsx
+++ b/reports/plans/noirs-boxes/2026-W19/2026-W19-0504-0510.xlsx
@@ -5,18 +5,17 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="TopicResearch" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="OwnHistory" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Frequency" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Schedule" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Metrics" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Meta" state="visible" r:id="rId9"/>
+    <sheet sheetId="2" name="Frequency" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Schedule" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Metrics" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Meta" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="86">
   <si>
     <t>platform</t>
   </si>
@@ -91,36 +90,6 @@
   </si>
   <si>
     <t>name the brand under test → drives engagement</t>
-  </si>
-  <si>
-    <t>caption_excerpt</t>
-  </si>
-  <si>
-    <t>repeatable_pattern</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/Y/</t>
-  </si>
-  <si>
-    <t>2026-04-15</t>
-  </si>
-  <si>
-    <t>PD vs QC — same wattage, different protocol. Here's why it matters.</t>
-  </si>
-  <si>
-    <t>technical-explainer</t>
-  </si>
-  <si>
-    <t>reel + 2-line caption</t>
-  </si>
-  <si>
-    <t>Same wattage, different protocol</t>
-  </si>
-  <si>
-    <t>educational hook on a confusion point repair shops face</t>
-  </si>
-  <si>
-    <t>lead with a 'same X different Y' contrast</t>
   </si>
   <si>
     <t>posts_per_week</t>
@@ -809,113 +778,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="30" customWidth="1"/>
-    <col min="11" max="11" width="40" customWidth="1"/>
-    <col min="12" max="13" width="50" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2">
-        <v>120</v>
-      </c>
-      <c r="E2">
-        <v>8</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>1800</v>
-      </c>
-      <c r="H2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -931,16 +793,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -951,30 +813,30 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B3">
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -983,7 +845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1007,143 +869,143 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="I2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="J2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="L2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="M2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="N2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="O2" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="G3" t="s">
         <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="J3" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L3" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" t="s">
+        <v>57</v>
+      </c>
+      <c r="O3" t="s">
         <v>67</v>
-      </c>
-      <c r="L3" t="s">
-        <v>68</v>
-      </c>
-      <c r="M3" t="s">
-        <v>67</v>
-      </c>
-      <c r="N3" t="s">
-        <v>67</v>
-      </c>
-      <c r="O3" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1152,7 +1014,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1168,28 +1030,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1198,7 +1060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1209,66 +1071,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>